<commit_message>
fix: tooltips now visible on hover - inlined CSS/JS to avoid CORS on file://
</commit_message>
<xml_diff>
--- a/Vonovia_Dashboard.xlsx
+++ b/Vonovia_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/08ec859eac6fe40e/ControllingDashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0911EDB5-7703-9444-BB60-64BDA88E5045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{0911EDB5-7703-9444-BB60-64BDA88E5045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCBBB33F-398C-D148-B776-B295B6816372}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{B42F3329-DB07-034F-B293-586B02AD4095}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="34">
   <si>
     <t>Jahr</t>
   </si>
@@ -155,6 +155,9 @@
   </si>
   <si>
     <t>Min. of Mitarbeiterzufriedenheit</t>
+  </si>
+  <si>
+    <t>a</t>
   </si>
 </sst>
 </file>
@@ -3825,59 +3828,47 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$4:$A$11</c:f>
+              <c:f>'.'!$A$4:$A$9</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$4:$B$11</c:f>
+              <c:f>'.'!$B$4:$B$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>43.1</c:v>
+                  <c:v>39.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>39.4</c:v>
+                  <c:v>45.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>45.4</c:v>
+                  <c:v>45.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>45.1</c:v>
+                  <c:v>47.3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>47.3</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>47.7</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>45.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4747,59 +4738,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$168:$A$175</c:f>
+              <c:f>'.'!$A$168:$A$173</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$168:$B$175</c:f>
+              <c:f>'.'!$B$168:$B$173</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>47.2</c:v>
+                  <c:v>39.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>39.5</c:v>
+                  <c:v>38.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>38.4</c:v>
+                  <c:v>33</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>33</c:v>
+                  <c:v>31.7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>31.7</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>31.2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>30.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5669,39 +5648,33 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$180:$A$187</c:f>
+              <c:f>'.'!$A$180:$A$185</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$180:$B$187</c:f>
+              <c:f>'.'!$B$180:$B$185</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -5715,13 +5688,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>0.75</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.77</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6199,59 +6166,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$209:$A$216</c:f>
+              <c:f>'.'!$A$209:$A$214</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$209:$B$216</c:f>
+              <c:f>'.'!$B$209:$B$214</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>47.8</c:v>
+                  <c:v>46.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>46.1</c:v>
+                  <c:v>40.1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>40.1</c:v>
+                  <c:v>51.3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>51.3</c:v>
+                  <c:v>51.7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>51.7</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>50.9</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>47.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9312,59 +9267,47 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$4:$A$11</c:f>
+              <c:f>'.'!$A$4:$A$9</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$4:$B$11</c:f>
+              <c:f>'.'!$B$4:$B$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>43.1</c:v>
+                  <c:v>39.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>39.4</c:v>
+                  <c:v>45.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>45.4</c:v>
+                  <c:v>45.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>45.1</c:v>
+                  <c:v>47.3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>47.3</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>47.7</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>45.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10150,59 +10093,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$32:$A$39</c:f>
+              <c:f>'.'!$A$32:$A$37</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$32:$B$39</c:f>
+              <c:f>'.'!$B$32:$B$37</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1760.1</c:v>
+                  <c:v>1909.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1909.8</c:v>
+                  <c:v>2254.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2254.4</c:v>
+                  <c:v>2606.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2606.1</c:v>
+                  <c:v>2583.8000000000002</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2583.8000000000002</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2641.8</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2800.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10963,59 +10894,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$52:$A$59</c:f>
+              <c:f>'.'!$A$52:$A$57</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$52:$B$59</c:f>
+              <c:f>'.'!$B$52:$B$57</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.29</c:v>
+                  <c:v>5.35</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.35</c:v>
+                  <c:v>2.2999999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.2999999999999998</c:v>
+                  <c:v>-0.66</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-0.66</c:v>
+                  <c:v>-7.34</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-7.34</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>-1.07</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>4.49</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11802,59 +11721,47 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$52:$A$59</c:f>
+              <c:f>'.'!$A$52:$A$57</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$52:$B$59</c:f>
+              <c:f>'.'!$B$52:$B$57</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.29</c:v>
+                  <c:v>5.35</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.35</c:v>
+                  <c:v>2.2999999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.2999999999999998</c:v>
+                  <c:v>-0.66</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-0.66</c:v>
+                  <c:v>-7.34</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-7.34</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>-1.07</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>4.49</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13033,59 +12940,47 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$69:$A$76</c:f>
+              <c:f>'.'!$A$69:$A$74</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$69:$B$76</c:f>
+              <c:f>'.'!$B$69:$B$74</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>61.2</c:v>
+                  <c:v>69.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>69.8</c:v>
+                  <c:v>74.3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>74.3</c:v>
+                  <c:v>75.599999999999994</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>75.599999999999994</c:v>
+                  <c:v>72.400000000000006</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>72.400000000000006</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>75.2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>76.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13876,59 +13771,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$92:$A$99</c:f>
+              <c:f>'.'!$A$92:$A$97</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$92:$B$99</c:f>
+              <c:f>'.'!$B$92:$B$97</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.6</c:v>
+                  <c:v>2.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.4</c:v>
+                  <c:v>2.2000000000000002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.2000000000000002</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -14715,58 +14598,46 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$107:$A$114</c:f>
+              <c:f>'.'!$A$107:$A$112</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$107:$B$114</c:f>
+              <c:f>'.'!$B$107:$B$112</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>3.9</c:v>
+                  <c:v>3.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.1</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>3.3</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>3.8</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>3.3</c:v>
-                </c:pt>
                 <c:pt idx="4">
-                  <c:v>3.8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>4.0999999999999996</c:v>
-                </c:pt>
-                <c:pt idx="6">
                   <c:v>4.0999999999999996</c:v>
                 </c:pt>
               </c:numCache>
@@ -15669,59 +15540,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$32:$A$39</c:f>
+              <c:f>'.'!$A$32:$A$37</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$32:$B$39</c:f>
+              <c:f>'.'!$B$32:$B$37</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1760.1</c:v>
+                  <c:v>1909.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1909.8</c:v>
+                  <c:v>2254.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2254.4</c:v>
+                  <c:v>2606.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2606.1</c:v>
+                  <c:v>2583.8000000000002</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2583.8000000000002</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2641.8</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2800.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -16475,59 +16334,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$117:$A$124</c:f>
+              <c:f>'.'!$A$117:$A$122</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$117:$B$124</c:f>
+              <c:f>'.'!$B$117:$B$122</c:f>
               <c:numCache>
                 <c:formatCode>#,##0\ "€"</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1971.1</c:v>
+                  <c:v>1935.9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1935.9</c:v>
+                  <c:v>2185.6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2185.6</c:v>
+                  <c:v>2266.3000000000002</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2266.3000000000002</c:v>
+                  <c:v>1527</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1527</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>1601</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1972.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -17314,59 +17161,47 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$135:$A$142</c:f>
+              <c:f>'.'!$A$135:$A$140</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$135:$B$142</c:f>
+              <c:f>'.'!$B$135:$B$140</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>12.2</c:v>
+                  <c:v>12.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12.1</c:v>
+                  <c:v>13.01</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>13.01</c:v>
+                  <c:v>12.86</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>12.86</c:v>
+                  <c:v>12.41</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>12.41</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>13.82</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>14.46</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -18152,59 +17987,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$150:$A$157</c:f>
+              <c:f>'.'!$A$150:$A$155</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$150:$B$157</c:f>
+              <c:f>'.'!$B$150:$B$155</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2092</c:v>
+                  <c:v>2088</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2088</c:v>
+                  <c:v>2200</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2200</c:v>
+                  <c:v>3749</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3749</c:v>
+                  <c:v>2460</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2460</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>3747</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2090</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -18990,59 +18813,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$168:$A$175</c:f>
+              <c:f>'.'!$A$168:$A$173</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$168:$B$175</c:f>
+              <c:f>'.'!$B$168:$B$173</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>47.2</c:v>
+                  <c:v>39.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>39.5</c:v>
+                  <c:v>38.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>38.4</c:v>
+                  <c:v>33</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>33</c:v>
+                  <c:v>31.7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>31.7</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>31.2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>30.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -19828,39 +19639,33 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$180:$A$187</c:f>
+              <c:f>'.'!$A$180:$A$185</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$180:$B$187</c:f>
+              <c:f>'.'!$B$180:$B$185</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -19874,13 +19679,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>0.75</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.77</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -20274,59 +20073,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$209:$A$216</c:f>
+              <c:f>'.'!$A$209:$A$214</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$209:$B$216</c:f>
+              <c:f>'.'!$B$209:$B$214</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>47.8</c:v>
+                  <c:v>46.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>46.1</c:v>
+                  <c:v>40.1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>40.1</c:v>
+                  <c:v>51.3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>51.3</c:v>
+                  <c:v>51.7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>51.7</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>50.9</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>47.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -21235,59 +21022,47 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$52:$A$59</c:f>
+              <c:f>'.'!$A$52:$A$57</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$52:$B$59</c:f>
+              <c:f>'.'!$B$52:$B$57</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.29</c:v>
+                  <c:v>5.35</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.35</c:v>
+                  <c:v>2.2999999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.2999999999999998</c:v>
+                  <c:v>-0.66</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-0.66</c:v>
+                  <c:v>-7.34</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-7.34</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>-1.07</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>4.49</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -22556,59 +22331,47 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$69:$A$76</c:f>
+              <c:f>'.'!$A$69:$A$74</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$69:$B$76</c:f>
+              <c:f>'.'!$B$69:$B$74</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>61.2</c:v>
+                  <c:v>69.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>69.8</c:v>
+                  <c:v>74.3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>74.3</c:v>
+                  <c:v>75.599999999999994</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>75.599999999999994</c:v>
+                  <c:v>72.400000000000006</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>72.400000000000006</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>75.2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>76.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -23491,59 +23254,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$92:$A$99</c:f>
+              <c:f>'.'!$A$92:$A$97</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$92:$B$99</c:f>
+              <c:f>'.'!$B$92:$B$97</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.6</c:v>
+                  <c:v>2.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.4</c:v>
+                  <c:v>2.2000000000000002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.2000000000000002</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -24420,58 +24171,46 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$107:$A$114</c:f>
+              <c:f>'.'!$A$107:$A$112</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$107:$B$114</c:f>
+              <c:f>'.'!$B$107:$B$112</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>3.9</c:v>
+                  <c:v>3.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.1</c:v>
+                  <c:v>3.8</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>3.3</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>3.8</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>3.3</c:v>
-                </c:pt>
                 <c:pt idx="4">
-                  <c:v>3.8</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>4.0999999999999996</c:v>
-                </c:pt>
-                <c:pt idx="6">
                   <c:v>4.0999999999999996</c:v>
                 </c:pt>
               </c:numCache>
@@ -25342,59 +25081,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$117:$A$124</c:f>
+              <c:f>'.'!$A$117:$A$122</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$117:$B$124</c:f>
+              <c:f>'.'!$B$117:$B$122</c:f>
               <c:numCache>
                 <c:formatCode>#,##0\ "€"</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1971.1</c:v>
+                  <c:v>1935.9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1935.9</c:v>
+                  <c:v>2185.6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2185.6</c:v>
+                  <c:v>2266.3000000000002</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2266.3000000000002</c:v>
+                  <c:v>1527</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1527</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>1601</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1972.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -26271,59 +25998,47 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$135:$A$142</c:f>
+              <c:f>'.'!$A$135:$A$140</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$135:$B$142</c:f>
+              <c:f>'.'!$B$135:$B$140</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>12.2</c:v>
+                  <c:v>12.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12.1</c:v>
+                  <c:v>13.01</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>13.01</c:v>
+                  <c:v>12.86</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>12.86</c:v>
+                  <c:v>12.41</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>12.41</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>13.82</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>14.46</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -27193,59 +26908,47 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$150:$A$157</c:f>
+              <c:f>'.'!$A$150:$A$155</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2019</c:v>
+                  <c:v>2020</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2020</c:v>
+                  <c:v>2021</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2021</c:v>
+                  <c:v>2022</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2022</c:v>
+                  <c:v>2023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2023</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>2024</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$150:$B$157</c:f>
+              <c:f>'.'!$B$150:$B$155</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2092</c:v>
+                  <c:v>2088</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2088</c:v>
+                  <c:v>2200</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2200</c:v>
+                  <c:v>3749</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3749</c:v>
+                  <c:v>2460</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2460</c:v>
-                </c:pt>
-                <c:pt idx="5">
                   <c:v>3747</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2090</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -42152,8 +41855,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="26737829" y="4014470"/>
-          <a:ext cx="2003541" cy="2863269"/>
+          <a:off x="26516083" y="4077466"/>
+          <a:ext cx="1989682" cy="2907366"/>
           <a:chOff x="6094931" y="736600"/>
           <a:chExt cx="1972109" cy="2929944"/>
         </a:xfrm>
@@ -42250,8 +41953,8 @@
             </xdr:nvSpPr>
             <xdr:spPr>
               <a:xfrm>
-                <a:off x="26880627" y="4122881"/>
-                <a:ext cx="1702743" cy="2683506"/>
+                <a:off x="26657893" y="4187546"/>
+                <a:ext cx="1690965" cy="2724835"/>
               </a:xfrm>
               <a:prstGeom prst="rect">
                 <a:avLst/>
@@ -42728,7 +42431,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>4624</xdr:colOff>
+      <xdr:colOff>4625</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>4553</xdr:rowOff>
     </xdr:to>
@@ -42766,7 +42469,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="8848965" y="5654591"/>
+              <a:off x="10391108" y="5654591"/>
               <a:ext cx="1799469" cy="2725914"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -43541,19 +43244,19 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0C6A04BC-1941-E145-9AD4-63F7AB7D8137}" name="PivotTable7" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
-  <location ref="A106:B114" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A106:B112" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -43574,10 +43277,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -43592,9 +43292,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -43724,19 +43421,19 @@
 
 <file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6D1407B9-D7EA-DD46-80D0-19DD7012609E}" name="PivotTable9" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="A134:B142" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A134:B140" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -43757,10 +43454,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -43775,9 +43469,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -43907,19 +43598,19 @@
 
 <file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{898BD313-1C04-0640-A33A-EBA664F923A2}" name="PivotTable3" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="A31:B39" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A31:B37" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -43940,10 +43631,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -43958,9 +43646,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -44090,19 +43775,19 @@
 
 <file path=xl/pivotTables/pivotTable12.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{55A28588-315F-7E47-BABA-8D570AA73DD4}" name="PivotTable8" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8">
-  <location ref="A116:B124" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A116:B122" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -44123,10 +43808,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -44141,9 +43823,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -44357,19 +44036,19 @@
 
 <file path=xl/pivotTables/pivotTable13.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C7101ABE-8B47-D84D-AB57-67B5E5546AA6}" name="PivotTable2" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
-  <location ref="A3:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -44390,10 +44069,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -44408,9 +44084,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -44540,19 +44213,19 @@
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C9C10335-3997-204F-94E0-80817EED75F1}" name="PivotTable14" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
-  <location ref="A208:B216" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A208:B214" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -44573,10 +44246,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -44591,9 +44261,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -44733,19 +44400,19 @@
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B3D7ADE2-C5AE-E84B-A075-E5FD8410E97E}" name="PivotTable12" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
-  <location ref="A179:B187" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A179:B185" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -44766,10 +44433,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -44784,9 +44448,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -44916,19 +44577,19 @@
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{36C26D69-C1AA-3C46-BDCF-5EACA398527D}" name="PivotTable11" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="A167:B175" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A167:B173" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -44949,10 +44610,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -44967,9 +44625,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -45099,19 +44754,19 @@
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{76DE73AF-06A4-7E49-B144-24717622BB4D}" name="PivotTable6" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="A91:B99" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A91:B97" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -45132,10 +44787,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -45150,9 +44802,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -45282,19 +44931,19 @@
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CAB156BD-6025-1947-8D45-C0E84232AD70}" name="PivotTable10" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="A149:B157" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A149:B155" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -45315,10 +44964,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -45333,9 +44979,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -45465,19 +45108,19 @@
 
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{742C156D-3F2A-0343-946F-4E6CC6909EF4}" name="PivotTable5" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
-  <location ref="A68:B76" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A68:B74" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -45498,10 +45141,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -45516,9 +45156,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -45648,19 +45285,19 @@
 
 <file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B3A72949-D391-9944-B7B5-88F38296042D}" name="PivotTable4" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
-  <location ref="A51:B59" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A51:B57" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item x="0"/>
+        <item h="1" x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
-        <item m="1" x="7"/>
-        <item m="1" x="8"/>
+        <item h="1" x="6"/>
+        <item h="1" m="1" x="7"/>
+        <item h="1" m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -45681,10 +45318,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="8">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="6">
     <i>
       <x v="1"/>
     </i>
@@ -45699,9 +45333,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -45941,15 +45572,15 @@
   <data>
     <tabular pivotCacheId="1673180031">
       <items count="9">
-        <i x="0" s="1"/>
+        <i x="0"/>
         <i x="1" s="1"/>
         <i x="2" s="1"/>
         <i x="3" s="1"/>
         <i x="4" s="1"/>
         <i x="5" s="1"/>
-        <i x="6" s="1"/>
-        <i x="7" s="1" nd="1"/>
-        <i x="8" s="1" nd="1"/>
+        <i x="6"/>
+        <i x="7" nd="1"/>
+        <i x="8" nd="1"/>
       </items>
     </tabular>
   </data>
@@ -46313,12 +45944,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFA51C22-640F-DF42-AC73-03CB6BE63A38}">
-  <dimension ref="A1"/>
+  <dimension ref="AK48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="10.83203125" style="7"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="48" spans="37:37" x14ac:dyDescent="0.2">
+      <c r="AK48" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
@@ -46713,11 +46350,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{256A9D5D-D368-E045-B17B-964952BB875E}">
-  <dimension ref="A3:AC216"/>
+  <dimension ref="A3:AC214"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="8" width="5.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.33203125" bestFit="1" customWidth="1"/>
@@ -46742,50 +46379,50 @@
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B4" s="6">
-        <v>43.1</v>
+        <v>39.4</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A5" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B5" s="6">
-        <v>39.4</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B6" s="6">
-        <v>45.4</v>
+        <v>45.1</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A7" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B7" s="6">
-        <v>45.1</v>
+        <v>47.3</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A8" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B8" s="6">
-        <v>47.3</v>
+        <v>47.7</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A9" s="5">
-        <v>2024</v>
+      <c r="A9" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B9" s="6">
-        <v>47.7</v>
+        <v>224.89999999999998</v>
       </c>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
@@ -46809,12 +46446,6 @@
       <c r="AC9" s="7"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A10" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B10" s="6">
-        <v>45.4</v>
-      </c>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
@@ -46837,12 +46468,6 @@
       <c r="AC10" s="7"/>
     </row>
     <row r="11" spans="1:29" ht="93" x14ac:dyDescent="0.2">
-      <c r="A11" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="6">
-        <v>313.39999999999998</v>
-      </c>
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
@@ -47312,10 +46937,10 @@
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A32" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B32" s="6">
-        <v>1760.1</v>
+        <v>1909.8</v>
       </c>
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
@@ -47340,10 +46965,10 @@
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A33" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B33" s="6">
-        <v>1909.8</v>
+        <v>2254.4</v>
       </c>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
@@ -47368,10 +46993,10 @@
     </row>
     <row r="34" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A34" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B34" s="6">
-        <v>2254.4</v>
+        <v>2606.1</v>
       </c>
       <c r="J34" s="7"/>
       <c r="K34" s="7"/>
@@ -47396,10 +47021,10 @@
     </row>
     <row r="35" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A35" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B35" s="6">
-        <v>2606.1</v>
+        <v>2583.8000000000002</v>
       </c>
       <c r="J35" s="7"/>
       <c r="K35" s="7"/>
@@ -47424,10 +47049,10 @@
     </row>
     <row r="36" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A36" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B36" s="6">
-        <v>2583.8000000000002</v>
+        <v>2641.8</v>
       </c>
       <c r="J36" s="7"/>
       <c r="K36" s="7"/>
@@ -47451,11 +47076,11 @@
       <c r="AC36" s="7"/>
     </row>
     <row r="37" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A37" s="5">
-        <v>2024</v>
+      <c r="A37" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B37" s="6">
-        <v>2641.8</v>
+        <v>11995.899999999998</v>
       </c>
       <c r="J37" s="7"/>
       <c r="K37" s="7"/>
@@ -47479,12 +47104,6 @@
       <c r="AC37" s="7"/>
     </row>
     <row r="38" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A38" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B38" s="6">
-        <v>2800.8</v>
-      </c>
       <c r="J38" s="7"/>
       <c r="K38" s="7"/>
       <c r="L38" s="7"/>
@@ -47507,12 +47126,6 @@
       <c r="AC38" s="7"/>
     </row>
     <row r="39" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A39" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B39" s="6">
-        <v>16556.8</v>
-      </c>
       <c r="J39" s="7"/>
       <c r="K39" s="7"/>
       <c r="L39" s="7"/>
@@ -47806,10 +47419,10 @@
     </row>
     <row r="52" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A52" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B52" s="6">
-        <v>2.29</v>
+        <v>5.35</v>
       </c>
       <c r="J52" s="7"/>
       <c r="K52" s="7"/>
@@ -47834,10 +47447,10 @@
     </row>
     <row r="53" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A53" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B53" s="6">
-        <v>5.35</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="J53" s="7"/>
       <c r="K53" s="7"/>
@@ -47862,10 +47475,10 @@
     </row>
     <row r="54" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A54" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B54" s="6">
-        <v>2.2999999999999998</v>
+        <v>-0.66</v>
       </c>
       <c r="J54" s="7"/>
       <c r="K54" s="7"/>
@@ -47890,10 +47503,10 @@
     </row>
     <row r="55" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A55" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B55" s="6">
-        <v>-0.66</v>
+        <v>-7.34</v>
       </c>
       <c r="J55" s="7"/>
       <c r="K55" s="7"/>
@@ -47918,10 +47531,10 @@
     </row>
     <row r="56" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A56" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B56" s="6">
-        <v>-7.34</v>
+        <v>-1.07</v>
       </c>
       <c r="J56" s="7"/>
       <c r="K56" s="7"/>
@@ -47945,11 +47558,11 @@
       <c r="AC56" s="7"/>
     </row>
     <row r="57" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A57" s="5">
-        <v>2024</v>
+      <c r="A57" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B57" s="6">
-        <v>-1.07</v>
+        <v>-1.4200000000000006</v>
       </c>
       <c r="J57" s="7"/>
       <c r="K57" s="7"/>
@@ -47973,12 +47586,6 @@
       <c r="AC57" s="7"/>
     </row>
     <row r="58" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A58" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B58" s="6">
-        <v>4.49</v>
-      </c>
       <c r="J58" s="7"/>
       <c r="K58" s="7"/>
       <c r="L58" s="7"/>
@@ -48001,12 +47608,6 @@
       <c r="AC58" s="7"/>
     </row>
     <row r="59" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A59" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B59" s="6">
-        <v>5.3599999999999994</v>
-      </c>
       <c r="J59" s="7"/>
       <c r="K59" s="7"/>
       <c r="L59" s="7"/>
@@ -48126,66 +47727,50 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B69" s="6">
-        <v>61.2</v>
+        <v>69.8</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B70" s="6">
-        <v>69.8</v>
+        <v>74.3</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B71" s="6">
-        <v>74.3</v>
+        <v>75.599999999999994</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B72" s="6">
-        <v>75.599999999999994</v>
+        <v>72.400000000000006</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B73" s="6">
-        <v>72.400000000000006</v>
+        <v>75.2</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A74" s="5">
-        <v>2024</v>
+      <c r="A74" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B74" s="6">
-        <v>75.2</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A75" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B75" s="6">
-        <v>76.5</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A76" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B76" s="6">
-        <v>504.99999999999994</v>
+        <v>367.3</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
@@ -48198,31 +47783,31 @@
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B92" s="6">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B93" s="6">
-        <v>2.4</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B94" s="6">
-        <v>2.2000000000000002</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B95" s="6">
         <v>2</v>
@@ -48230,34 +47815,18 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B96" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A97" s="5">
-        <v>2024</v>
+      <c r="A97" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B97" s="6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A98" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B98" s="6">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A99" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B99" s="6">
-        <v>15.299999999999999</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
@@ -48270,66 +47839,50 @@
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B107" s="6">
-        <v>3.9</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B108" s="6">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B109" s="6">
-        <v>3.8</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A110" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B110" s="6">
-        <v>3.3</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A111" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B111" s="6">
-        <v>3.8</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A112" s="5">
-        <v>2024</v>
+      <c r="A112" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B112" s="6">
-        <v>4.0999999999999996</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A113" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B113" s="6">
-        <v>4.0999999999999996</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A114" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B114" s="6">
-        <v>26.1</v>
+        <v>18.100000000000001</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
@@ -48342,66 +47895,50 @@
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A117" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B117" s="4">
-        <v>1971.1</v>
+        <v>1935.9</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A118" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B118" s="4">
-        <v>1935.9</v>
+        <v>2185.6</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A119" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B119" s="4">
-        <v>2185.6</v>
+        <v>2266.3000000000002</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A120" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B120" s="4">
-        <v>2266.3000000000002</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A121" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B121" s="4">
-        <v>1527</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A122" s="5">
-        <v>2024</v>
+      <c r="A122" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B122" s="4">
-        <v>1601</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A123" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B123" s="4">
-        <v>1972.7</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A124" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B124" s="4">
-        <v>13459.600000000002</v>
+        <v>9515.7999999999993</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.2">
@@ -48414,66 +47951,50 @@
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A135" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B135" s="6">
-        <v>12.2</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A136" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B136" s="6">
-        <v>12.1</v>
+        <v>13.01</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A137" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B137" s="6">
-        <v>13.01</v>
+        <v>12.86</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A138" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B138" s="6">
-        <v>12.86</v>
+        <v>12.41</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A139" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B139" s="6">
-        <v>12.41</v>
+        <v>13.82</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A140" s="5">
-        <v>2024</v>
+      <c r="A140" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B140" s="6">
-        <v>13.82</v>
-      </c>
-    </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A141" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B141" s="6">
-        <v>14.46</v>
-      </c>
-    </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A142" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B142" s="6">
-        <v>90.860000000000014</v>
+        <v>64.199999999999989</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.2">
@@ -48486,66 +48007,50 @@
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A150" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B150" s="6">
-        <v>2092</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A151" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B151" s="6">
-        <v>2088</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A152" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B152" s="6">
-        <v>2200</v>
+        <v>3749</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A153" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B153" s="6">
-        <v>3749</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A154" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B154" s="6">
-        <v>2460</v>
+        <v>3747</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A155" s="5">
-        <v>2024</v>
+      <c r="A155" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B155" s="6">
-        <v>3747</v>
-      </c>
-    </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A156" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B156" s="6">
-        <v>2090</v>
-      </c>
-    </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A157" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B157" s="6">
-        <v>18426</v>
+        <v>14244</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.2">
@@ -48558,66 +48063,50 @@
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A168" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B168" s="6">
-        <v>47.2</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A169" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B169" s="6">
-        <v>39.5</v>
+        <v>38.4</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A170" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B170" s="6">
-        <v>38.4</v>
+        <v>33</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A171" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B171" s="6">
-        <v>33</v>
+        <v>31.7</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A172" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B172" s="6">
-        <v>31.7</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A173" s="5">
-        <v>2024</v>
+      <c r="A173" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B173" s="6">
-        <v>31.2</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A174" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B174" s="6">
-        <v>30.7</v>
-      </c>
-    </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A175" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B175" s="6">
-        <v>251.69999999999996</v>
+        <v>173.79999999999998</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.2">
@@ -48630,7 +48119,7 @@
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A180" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B180" s="6">
         <v>0</v>
@@ -48638,7 +48127,7 @@
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A181" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B181" s="6">
         <v>0</v>
@@ -48646,7 +48135,7 @@
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A182" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B182" s="6">
         <v>0</v>
@@ -48654,7 +48143,7 @@
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A183" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B183" s="6">
         <v>0</v>
@@ -48662,33 +48151,17 @@
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A184" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B184" s="6">
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A185" s="5">
-        <v>2024</v>
+      <c r="A185" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B185" s="6">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A186" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B186" s="6">
-        <v>0.77</v>
-      </c>
-    </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A187" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B187" s="6">
         <v>0</v>
       </c>
     </row>
@@ -48766,66 +48239,50 @@
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A209" s="5">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B209" s="6">
-        <v>47.8</v>
+        <v>46.1</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A210" s="5">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B210" s="6">
-        <v>46.1</v>
+        <v>40.1</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A211" s="5">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B211" s="6">
-        <v>40.1</v>
+        <v>51.3</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A212" s="5">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B212" s="6">
-        <v>51.3</v>
+        <v>51.7</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A213" s="5">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B213" s="6">
-        <v>51.7</v>
+        <v>50.9</v>
       </c>
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A214" s="5">
-        <v>2024</v>
+      <c r="A214" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="B214" s="6">
-        <v>50.9</v>
-      </c>
-    </row>
-    <row r="215" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A215" s="5">
-        <v>2025</v>
-      </c>
-      <c r="B215" s="6">
-        <v>47.8</v>
-      </c>
-    </row>
-    <row r="216" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A216" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B216" s="6">
-        <v>335.7</v>
+        <v>240.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: interactive year filter with crisis preset for presentation
- Toggle individual years on/off across all charts
- 'Krise 2022-2023' preset isolates crisis period (2021-2024)
- 'Alle' button resets to full view
- 'Ziel 2028' toggle to show/hide targets
- Charts rebuild dynamically on filter change
</commit_message>
<xml_diff>
--- a/Vonovia_Dashboard.xlsx
+++ b/Vonovia_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/08ec859eac6fe40e/ControllingDashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{0911EDB5-7703-9444-BB60-64BDA88E5045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCBBB33F-398C-D148-B776-B295B6816372}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{0911EDB5-7703-9444-BB60-64BDA88E5045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40E7BAAE-24CA-4049-9CF9-685C1F462AC0}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{B42F3329-DB07-034F-B293-586B02AD4095}"/>
   </bookViews>
@@ -3828,47 +3828,59 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$4:$A$9</c:f>
+              <c:f>'.'!$A$4:$A$11</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$4:$B$9</c:f>
+              <c:f>'.'!$B$4:$B$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>43.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>39.4</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>45.4</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>45.1</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>47.3</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>47.7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>45.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4738,47 +4750,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$168:$A$173</c:f>
+              <c:f>'.'!$A$168:$A$175</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$168:$B$173</c:f>
+              <c:f>'.'!$B$168:$B$175</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>47.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>39.5</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>38.4</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>33</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>31.7</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>31.2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5648,33 +5672,39 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$180:$A$185</c:f>
+              <c:f>'.'!$A$180:$A$187</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$180:$B$185</c:f>
+              <c:f>'.'!$B$180:$B$187</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -5688,7 +5718,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.77</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6166,47 +6202,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$209:$A$214</c:f>
+              <c:f>'.'!$A$209:$A$216</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$209:$B$214</c:f>
+              <c:f>'.'!$B$209:$B$216</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>47.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>46.1</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>40.1</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>51.3</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>51.7</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>50.9</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>47.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9267,47 +9315,59 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$4:$A$9</c:f>
+              <c:f>'.'!$A$4:$A$11</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$4:$B$9</c:f>
+              <c:f>'.'!$B$4:$B$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>43.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>39.4</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>45.4</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>45.1</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>47.3</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>47.7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>45.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10093,47 +10153,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$32:$A$37</c:f>
+              <c:f>'.'!$A$32:$A$39</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$32:$B$37</c:f>
+              <c:f>'.'!$B$32:$B$39</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>1760.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1909.8</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2254.4</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2606.1</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2583.8000000000002</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2641.8</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2800.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10894,47 +10966,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$52:$A$57</c:f>
+              <c:f>'.'!$A$52:$A$59</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$52:$B$57</c:f>
+              <c:f>'.'!$B$52:$B$59</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2.29</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>5.35</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2.2999999999999998</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>-0.66</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>-7.34</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>-1.07</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.49</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11721,47 +11805,59 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$52:$A$57</c:f>
+              <c:f>'.'!$A$52:$A$59</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$52:$B$57</c:f>
+              <c:f>'.'!$B$52:$B$59</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2.29</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>5.35</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2.2999999999999998</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>-0.66</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>-7.34</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>-1.07</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.49</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12940,47 +13036,59 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$69:$A$74</c:f>
+              <c:f>'.'!$A$69:$A$76</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$69:$B$74</c:f>
+              <c:f>'.'!$B$69:$B$76</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>61.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>69.8</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>74.3</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>75.599999999999994</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>72.400000000000006</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>75.2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>76.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13771,47 +13879,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$92:$A$97</c:f>
+              <c:f>'.'!$A$92:$A$99</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$92:$B$97</c:f>
+              <c:f>'.'!$B$92:$B$99</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2.6</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2.4</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2.2000000000000002</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -14598,46 +14718,58 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$107:$A$112</c:f>
+              <c:f>'.'!$A$107:$A$114</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$107:$B$112</c:f>
+              <c:f>'.'!$B$107:$B$114</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>3.9</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>3.1</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>3.8</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>3.3</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>3.8</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
+                  <c:v>4.0999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>4.0999999999999996</c:v>
                 </c:pt>
               </c:numCache>
@@ -15540,47 +15672,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$32:$A$37</c:f>
+              <c:f>'.'!$A$32:$A$39</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$32:$B$37</c:f>
+              <c:f>'.'!$B$32:$B$39</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>1760.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1909.8</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2254.4</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2606.1</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2583.8000000000002</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2641.8</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2800.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -16334,47 +16478,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$117:$A$122</c:f>
+              <c:f>'.'!$A$117:$A$124</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$117:$B$122</c:f>
+              <c:f>'.'!$B$117:$B$124</c:f>
               <c:numCache>
                 <c:formatCode>#,##0\ "€"</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>1971.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1935.9</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2185.6</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2266.3000000000002</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>1527</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>1601</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1972.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -17161,47 +17317,59 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$135:$A$140</c:f>
+              <c:f>'.'!$A$135:$A$142</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$135:$B$140</c:f>
+              <c:f>'.'!$B$135:$B$142</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>12.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>12.1</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>13.01</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>12.86</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>12.41</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>13.82</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>14.46</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -17987,47 +18155,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$150:$A$155</c:f>
+              <c:f>'.'!$A$150:$A$157</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$150:$B$155</c:f>
+              <c:f>'.'!$B$150:$B$157</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2092</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2088</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2200</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>3749</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2460</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>3747</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2090</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -18813,47 +18993,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$168:$A$173</c:f>
+              <c:f>'.'!$A$168:$A$175</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$168:$B$173</c:f>
+              <c:f>'.'!$B$168:$B$175</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>47.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>39.5</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>38.4</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>33</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>31.7</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>31.2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -19639,33 +19831,39 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$180:$A$185</c:f>
+              <c:f>'.'!$A$180:$A$187</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$180:$B$185</c:f>
+              <c:f>'.'!$B$180:$B$187</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -19679,7 +19877,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.77</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -20073,47 +20277,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$209:$A$214</c:f>
+              <c:f>'.'!$A$209:$A$216</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$209:$B$214</c:f>
+              <c:f>'.'!$B$209:$B$216</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>47.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>46.1</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>40.1</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>51.3</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>51.7</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>50.9</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>47.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -21022,47 +21238,59 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$52:$A$57</c:f>
+              <c:f>'.'!$A$52:$A$59</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$52:$B$57</c:f>
+              <c:f>'.'!$B$52:$B$59</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2.29</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>5.35</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2.2999999999999998</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>-0.66</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>-7.34</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>-1.07</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.49</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -22331,47 +22559,59 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$69:$A$74</c:f>
+              <c:f>'.'!$A$69:$A$76</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$69:$B$74</c:f>
+              <c:f>'.'!$B$69:$B$76</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>61.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>69.8</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>74.3</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>75.599999999999994</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>72.400000000000006</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>75.2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>76.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -23254,47 +23494,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$92:$A$97</c:f>
+              <c:f>'.'!$A$92:$A$99</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$92:$B$97</c:f>
+              <c:f>'.'!$B$92:$B$99</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2.6</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2.4</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2.2000000000000002</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -24171,46 +24423,58 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$107:$A$112</c:f>
+              <c:f>'.'!$A$107:$A$114</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$107:$B$112</c:f>
+              <c:f>'.'!$B$107:$B$114</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>3.9</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>3.1</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>3.8</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>3.3</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>3.8</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
+                  <c:v>4.0999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>4.0999999999999996</c:v>
                 </c:pt>
               </c:numCache>
@@ -25081,47 +25345,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$117:$A$122</c:f>
+              <c:f>'.'!$A$117:$A$124</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$117:$B$122</c:f>
+              <c:f>'.'!$B$117:$B$124</c:f>
               <c:numCache>
                 <c:formatCode>#,##0\ "€"</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>1971.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1935.9</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2185.6</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2266.3000000000002</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>1527</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>1601</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1972.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -25998,47 +26274,59 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$135:$A$140</c:f>
+              <c:f>'.'!$A$135:$A$142</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$135:$B$140</c:f>
+              <c:f>'.'!$B$135:$B$142</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>12.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>12.1</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>13.01</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>12.86</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>12.41</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>13.82</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>14.46</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -26908,47 +27196,59 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>'.'!$A$150:$A$155</c:f>
+              <c:f>'.'!$A$150:$A$157</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2019</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2020</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2021</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2022</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2023</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2025</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'.'!$B$150:$B$155</c:f>
+              <c:f>'.'!$B$150:$B$157</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2092</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2088</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2200</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>3749</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2460</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>3747</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2090</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -43244,19 +43544,19 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0C6A04BC-1941-E145-9AD4-63F7AB7D8137}" name="PivotTable7" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
-  <location ref="A106:B112" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A106:B114" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -43277,7 +43577,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -43292,6 +43595,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -43421,19 +43727,19 @@
 
 <file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6D1407B9-D7EA-DD46-80D0-19DD7012609E}" name="PivotTable9" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="A134:B140" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A134:B142" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -43454,7 +43760,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -43469,6 +43778,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -43598,19 +43910,19 @@
 
 <file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{898BD313-1C04-0640-A33A-EBA664F923A2}" name="PivotTable3" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="A31:B37" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A31:B39" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -43631,7 +43943,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -43646,6 +43961,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -43775,19 +44093,19 @@
 
 <file path=xl/pivotTables/pivotTable12.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{55A28588-315F-7E47-BABA-8D570AA73DD4}" name="PivotTable8" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8">
-  <location ref="A116:B122" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A116:B124" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -43808,7 +44126,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -43823,6 +44144,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -44036,19 +44360,19 @@
 
 <file path=xl/pivotTables/pivotTable13.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C7101ABE-8B47-D84D-AB57-67B5E5546AA6}" name="PivotTable2" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
-  <location ref="A3:B9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:B11" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -44069,7 +44393,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -44084,6 +44411,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -44213,19 +44543,19 @@
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C9C10335-3997-204F-94E0-80817EED75F1}" name="PivotTable14" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
-  <location ref="A208:B214" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A208:B216" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -44246,7 +44576,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -44261,6 +44594,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -44400,19 +44736,19 @@
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B3D7ADE2-C5AE-E84B-A075-E5FD8410E97E}" name="PivotTable12" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
-  <location ref="A179:B185" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A179:B187" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -44433,7 +44769,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -44448,6 +44787,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -44577,19 +44919,19 @@
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{36C26D69-C1AA-3C46-BDCF-5EACA398527D}" name="PivotTable11" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="A167:B173" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A167:B175" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -44610,7 +44952,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -44625,6 +44970,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -44754,19 +45102,19 @@
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{76DE73AF-06A4-7E49-B144-24717622BB4D}" name="PivotTable6" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="A91:B97" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A91:B99" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -44787,7 +45135,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -44802,6 +45153,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -44931,19 +45285,19 @@
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CAB156BD-6025-1947-8D45-C0E84232AD70}" name="PivotTable10" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="A149:B155" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A149:B157" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -44964,7 +45318,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -44979,6 +45336,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -45108,19 +45468,19 @@
 
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{742C156D-3F2A-0343-946F-4E6CC6909EF4}" name="PivotTable5" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
-  <location ref="A68:B74" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A68:B76" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -45141,7 +45501,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -45156,6 +45519,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -45285,19 +45651,19 @@
 
 <file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B3A72949-D391-9944-B7B5-88F38296042D}" name="PivotTable4" cacheId="105" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
-  <location ref="A51:B57" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A51:B59" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" showAll="0">
       <items count="10">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" m="1" x="7"/>
-        <item h="1" m="1" x="8"/>
+        <item x="6"/>
+        <item m="1" x="7"/>
+        <item m="1" x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -45318,7 +45684,10 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="6">
+  <rowItems count="8">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
     </i>
@@ -45333,6 +45702,9 @@
     </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -45572,15 +45944,15 @@
   <data>
     <tabular pivotCacheId="1673180031">
       <items count="9">
-        <i x="0"/>
+        <i x="0" s="1"/>
         <i x="1" s="1"/>
         <i x="2" s="1"/>
         <i x="3" s="1"/>
         <i x="4" s="1"/>
         <i x="5" s="1"/>
-        <i x="6"/>
-        <i x="7" nd="1"/>
-        <i x="8" nd="1"/>
+        <i x="6" s="1"/>
+        <i x="7" s="1" nd="1"/>
+        <i x="8" s="1" nd="1"/>
       </items>
     </tabular>
   </data>
@@ -46350,7 +46722,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{256A9D5D-D368-E045-B17B-964952BB875E}">
-  <dimension ref="A3:AC214"/>
+  <dimension ref="A3:AC216"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" bestFit="1" customWidth="1"/>
@@ -46379,50 +46751,50 @@
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B4" s="6">
-        <v>39.4</v>
+        <v>43.1</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A5" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B5" s="6">
-        <v>45.4</v>
+        <v>39.4</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B6" s="6">
-        <v>45.1</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A7" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B7" s="6">
-        <v>47.3</v>
+        <v>45.1</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A8" s="5">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B8" s="6">
-        <v>47.7</v>
+        <v>47.3</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
-        <v>16</v>
+      <c r="A9" s="5">
+        <v>2024</v>
       </c>
       <c r="B9" s="6">
-        <v>224.89999999999998</v>
+        <v>47.7</v>
       </c>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
@@ -46446,6 +46818,12 @@
       <c r="AC9" s="7"/>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A10" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B10" s="6">
+        <v>45.4</v>
+      </c>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
@@ -46468,6 +46846,12 @@
       <c r="AC10" s="7"/>
     </row>
     <row r="11" spans="1:29" ht="93" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="6">
+        <v>313.39999999999998</v>
+      </c>
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
@@ -46937,10 +47321,10 @@
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A32" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B32" s="6">
-        <v>1909.8</v>
+        <v>1760.1</v>
       </c>
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
@@ -46965,10 +47349,10 @@
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A33" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B33" s="6">
-        <v>2254.4</v>
+        <v>1909.8</v>
       </c>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
@@ -46993,10 +47377,10 @@
     </row>
     <row r="34" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A34" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B34" s="6">
-        <v>2606.1</v>
+        <v>2254.4</v>
       </c>
       <c r="J34" s="7"/>
       <c r="K34" s="7"/>
@@ -47021,10 +47405,10 @@
     </row>
     <row r="35" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A35" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B35" s="6">
-        <v>2583.8000000000002</v>
+        <v>2606.1</v>
       </c>
       <c r="J35" s="7"/>
       <c r="K35" s="7"/>
@@ -47049,10 +47433,10 @@
     </row>
     <row r="36" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A36" s="5">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B36" s="6">
-        <v>2641.8</v>
+        <v>2583.8000000000002</v>
       </c>
       <c r="J36" s="7"/>
       <c r="K36" s="7"/>
@@ -47076,11 +47460,11 @@
       <c r="AC36" s="7"/>
     </row>
     <row r="37" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A37" s="5" t="s">
-        <v>16</v>
+      <c r="A37" s="5">
+        <v>2024</v>
       </c>
       <c r="B37" s="6">
-        <v>11995.899999999998</v>
+        <v>2641.8</v>
       </c>
       <c r="J37" s="7"/>
       <c r="K37" s="7"/>
@@ -47104,6 +47488,12 @@
       <c r="AC37" s="7"/>
     </row>
     <row r="38" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A38" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B38" s="6">
+        <v>2800.8</v>
+      </c>
       <c r="J38" s="7"/>
       <c r="K38" s="7"/>
       <c r="L38" s="7"/>
@@ -47126,6 +47516,12 @@
       <c r="AC38" s="7"/>
     </row>
     <row r="39" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A39" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B39" s="6">
+        <v>16556.8</v>
+      </c>
       <c r="J39" s="7"/>
       <c r="K39" s="7"/>
       <c r="L39" s="7"/>
@@ -47419,10 +47815,10 @@
     </row>
     <row r="52" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A52" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B52" s="6">
-        <v>5.35</v>
+        <v>2.29</v>
       </c>
       <c r="J52" s="7"/>
       <c r="K52" s="7"/>
@@ -47447,10 +47843,10 @@
     </row>
     <row r="53" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A53" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B53" s="6">
-        <v>2.2999999999999998</v>
+        <v>5.35</v>
       </c>
       <c r="J53" s="7"/>
       <c r="K53" s="7"/>
@@ -47475,10 +47871,10 @@
     </row>
     <row r="54" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A54" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B54" s="6">
-        <v>-0.66</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="J54" s="7"/>
       <c r="K54" s="7"/>
@@ -47503,10 +47899,10 @@
     </row>
     <row r="55" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A55" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B55" s="6">
-        <v>-7.34</v>
+        <v>-0.66</v>
       </c>
       <c r="J55" s="7"/>
       <c r="K55" s="7"/>
@@ -47531,10 +47927,10 @@
     </row>
     <row r="56" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A56" s="5">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B56" s="6">
-        <v>-1.07</v>
+        <v>-7.34</v>
       </c>
       <c r="J56" s="7"/>
       <c r="K56" s="7"/>
@@ -47558,11 +47954,11 @@
       <c r="AC56" s="7"/>
     </row>
     <row r="57" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A57" s="5" t="s">
-        <v>16</v>
+      <c r="A57" s="5">
+        <v>2024</v>
       </c>
       <c r="B57" s="6">
-        <v>-1.4200000000000006</v>
+        <v>-1.07</v>
       </c>
       <c r="J57" s="7"/>
       <c r="K57" s="7"/>
@@ -47586,6 +47982,12 @@
       <c r="AC57" s="7"/>
     </row>
     <row r="58" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A58" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B58" s="6">
+        <v>4.49</v>
+      </c>
       <c r="J58" s="7"/>
       <c r="K58" s="7"/>
       <c r="L58" s="7"/>
@@ -47608,6 +48010,12 @@
       <c r="AC58" s="7"/>
     </row>
     <row r="59" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A59" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B59" s="6">
+        <v>5.3599999999999994</v>
+      </c>
       <c r="J59" s="7"/>
       <c r="K59" s="7"/>
       <c r="L59" s="7"/>
@@ -47727,50 +48135,66 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B69" s="6">
-        <v>69.8</v>
+        <v>61.2</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B70" s="6">
-        <v>74.3</v>
+        <v>69.8</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B71" s="6">
-        <v>75.599999999999994</v>
+        <v>74.3</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B72" s="6">
-        <v>72.400000000000006</v>
+        <v>75.599999999999994</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" s="5">
+        <v>2023</v>
+      </c>
+      <c r="B73" s="6">
+        <v>72.400000000000006</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" s="5">
         <v>2024</v>
       </c>
-      <c r="B73" s="6">
+      <c r="B74" s="6">
         <v>75.2</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A74" s="5" t="s">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B75" s="6">
+        <v>76.5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B74" s="6">
-        <v>367.3</v>
+      <c r="B76" s="6">
+        <v>504.99999999999994</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
@@ -47783,31 +48207,31 @@
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B92" s="6">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B93" s="6">
-        <v>2.2000000000000002</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B94" s="6">
-        <v>2</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B95" s="6">
         <v>2</v>
@@ -47815,18 +48239,34 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" s="5">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B96" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A97" s="5" t="s">
+      <c r="A97" s="5">
+        <v>2024</v>
+      </c>
+      <c r="B97" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A98" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B98" s="6">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A99" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B97" s="6">
-        <v>10.6</v>
+      <c r="B99" s="6">
+        <v>15.299999999999999</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
@@ -47839,50 +48279,66 @@
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B107" s="6">
-        <v>3.1</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B108" s="6">
-        <v>3.8</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B109" s="6">
-        <v>3.3</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A110" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B110" s="6">
-        <v>3.8</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A111" s="5">
+        <v>2023</v>
+      </c>
+      <c r="B111" s="6">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A112" s="5">
         <v>2024</v>
       </c>
-      <c r="B111" s="6">
+      <c r="B112" s="6">
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A112" s="5" t="s">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A113" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B113" s="6">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A114" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B112" s="6">
-        <v>18.100000000000001</v>
+      <c r="B114" s="6">
+        <v>26.1</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
@@ -47895,50 +48351,66 @@
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A117" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B117" s="4">
-        <v>1935.9</v>
+        <v>1971.1</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A118" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B118" s="4">
-        <v>2185.6</v>
+        <v>1935.9</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A119" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B119" s="4">
-        <v>2266.3000000000002</v>
+        <v>2185.6</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A120" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B120" s="4">
-        <v>1527</v>
+        <v>2266.3000000000002</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A121" s="5">
+        <v>2023</v>
+      </c>
+      <c r="B121" s="4">
+        <v>1527</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A122" s="5">
         <v>2024</v>
       </c>
-      <c r="B121" s="4">
+      <c r="B122" s="4">
         <v>1601</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A122" s="5" t="s">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A123" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B123" s="4">
+        <v>1972.7</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A124" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B122" s="4">
-        <v>9515.7999999999993</v>
+      <c r="B124" s="4">
+        <v>13459.600000000002</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.2">
@@ -47951,50 +48423,66 @@
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A135" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B135" s="6">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A136" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B136" s="6">
-        <v>13.01</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A137" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B137" s="6">
-        <v>12.86</v>
+        <v>13.01</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A138" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B138" s="6">
-        <v>12.41</v>
+        <v>12.86</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A139" s="5">
+        <v>2023</v>
+      </c>
+      <c r="B139" s="6">
+        <v>12.41</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A140" s="5">
         <v>2024</v>
       </c>
-      <c r="B139" s="6">
+      <c r="B140" s="6">
         <v>13.82</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A140" s="5" t="s">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A141" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B141" s="6">
+        <v>14.46</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A142" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B140" s="6">
-        <v>64.199999999999989</v>
+      <c r="B142" s="6">
+        <v>90.860000000000014</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.2">
@@ -48007,50 +48495,66 @@
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A150" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B150" s="6">
-        <v>2088</v>
+        <v>2092</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A151" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B151" s="6">
-        <v>2200</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A152" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B152" s="6">
-        <v>3749</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A153" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B153" s="6">
-        <v>2460</v>
+        <v>3749</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A154" s="5">
+        <v>2023</v>
+      </c>
+      <c r="B154" s="6">
+        <v>2460</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A155" s="5">
         <v>2024</v>
       </c>
-      <c r="B154" s="6">
+      <c r="B155" s="6">
         <v>3747</v>
       </c>
     </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A155" s="5" t="s">
+    <row r="156" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A156" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B156" s="6">
+        <v>2090</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A157" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B155" s="6">
-        <v>14244</v>
+      <c r="B157" s="6">
+        <v>18426</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.2">
@@ -48063,50 +48567,66 @@
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A168" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B168" s="6">
-        <v>39.5</v>
+        <v>47.2</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A169" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B169" s="6">
-        <v>38.4</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A170" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B170" s="6">
-        <v>33</v>
+        <v>38.4</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A171" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B171" s="6">
-        <v>31.7</v>
+        <v>33</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A172" s="5">
+        <v>2023</v>
+      </c>
+      <c r="B172" s="6">
+        <v>31.7</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A173" s="5">
         <v>2024</v>
       </c>
-      <c r="B172" s="6">
+      <c r="B173" s="6">
         <v>31.2</v>
       </c>
     </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A173" s="5" t="s">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A174" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B174" s="6">
+        <v>30.7</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A175" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B173" s="6">
-        <v>173.79999999999998</v>
+      <c r="B175" s="6">
+        <v>251.69999999999996</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.2">
@@ -48119,7 +48639,7 @@
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A180" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B180" s="6">
         <v>0</v>
@@ -48127,7 +48647,7 @@
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A181" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B181" s="6">
         <v>0</v>
@@ -48135,7 +48655,7 @@
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A182" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B182" s="6">
         <v>0</v>
@@ -48143,7 +48663,7 @@
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A183" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B183" s="6">
         <v>0</v>
@@ -48151,17 +48671,33 @@
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A184" s="5">
+        <v>2023</v>
+      </c>
+      <c r="B184" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A185" s="5">
         <v>2024</v>
       </c>
-      <c r="B184" s="6">
+      <c r="B185" s="6">
         <v>0.75</v>
       </c>
     </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A185" s="5" t="s">
+    <row r="186" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A186" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B186" s="6">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A187" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B185" s="6">
+      <c r="B187" s="6">
         <v>0</v>
       </c>
     </row>
@@ -48239,50 +48775,66 @@
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A209" s="5">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B209" s="6">
-        <v>46.1</v>
+        <v>47.8</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A210" s="5">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B210" s="6">
-        <v>40.1</v>
+        <v>46.1</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A211" s="5">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B211" s="6">
-        <v>51.3</v>
+        <v>40.1</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A212" s="5">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B212" s="6">
-        <v>51.7</v>
+        <v>51.3</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A213" s="5">
+        <v>2023</v>
+      </c>
+      <c r="B213" s="6">
+        <v>51.7</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A214" s="5">
         <v>2024</v>
       </c>
-      <c r="B213" s="6">
+      <c r="B214" s="6">
         <v>50.9</v>
       </c>
     </row>
-    <row r="214" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A214" s="5" t="s">
+    <row r="215" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A215" s="5">
+        <v>2025</v>
+      </c>
+      <c r="B215" s="6">
+        <v>47.8</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A216" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B214" s="6">
-        <v>240.1</v>
+      <c r="B216" s="6">
+        <v>335.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update maintSqm data and rebuild export files
</commit_message>
<xml_diff>
--- a/Vonovia_Dashboard.xlsx
+++ b/Vonovia_Dashboard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/08ec859eac6fe40e/ControllingDashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{0911EDB5-7703-9444-BB60-64BDA88E5045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40E7BAAE-24CA-4049-9CF9-685C1F462AC0}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{0911EDB5-7703-9444-BB60-64BDA88E5045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF323A7C-09FD-714B-A12A-8FC384D8CAFD}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{B42F3329-DB07-034F-B293-586B02AD4095}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{B42F3329-DB07-034F-B293-586B02AD4095}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard_" sheetId="3" r:id="rId1"/>
@@ -42155,8 +42155,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="26516083" y="4077466"/>
-          <a:ext cx="1989682" cy="2907366"/>
+          <a:off x="26619296" y="4109720"/>
+          <a:ext cx="1996132" cy="2929944"/>
           <a:chOff x="6094931" y="736600"/>
           <a:chExt cx="1972109" cy="2929944"/>
         </a:xfrm>
@@ -42253,8 +42253,8 @@
             </xdr:nvSpPr>
             <xdr:spPr>
               <a:xfrm>
-                <a:off x="26657893" y="4187546"/>
-                <a:ext cx="1690965" cy="2724835"/>
+                <a:off x="26761566" y="4220655"/>
+                <a:ext cx="1696446" cy="2745995"/>
               </a:xfrm>
               <a:prstGeom prst="rect">
                 <a:avLst/>
@@ -46431,7 +46431,7 @@
         <v>1971.1</v>
       </c>
       <c r="J2">
-        <v>12.2</v>
+        <v>19.02</v>
       </c>
       <c r="K2">
         <v>2092</v>
@@ -46472,7 +46472,7 @@
         <v>1935.9</v>
       </c>
       <c r="J3">
-        <v>12.1</v>
+        <v>22.31</v>
       </c>
       <c r="K3">
         <v>2088</v>
@@ -46516,7 +46516,7 @@
         <v>2185.6</v>
       </c>
       <c r="J4">
-        <v>13.01</v>
+        <v>26.17</v>
       </c>
       <c r="K4">
         <v>2200</v>
@@ -46557,7 +46557,7 @@
         <v>2266.3000000000002</v>
       </c>
       <c r="J5">
-        <v>12.86</v>
+        <v>24.81</v>
       </c>
       <c r="K5">
         <v>3749</v>
@@ -46601,7 +46601,7 @@
         <v>1527</v>
       </c>
       <c r="J6">
-        <v>12.41</v>
+        <v>21.03</v>
       </c>
       <c r="K6">
         <v>2460</v>
@@ -46645,7 +46645,7 @@
         <v>1601</v>
       </c>
       <c r="J7">
-        <v>13.82</v>
+        <v>22.46</v>
       </c>
       <c r="K7">
         <v>3747</v>
@@ -46689,7 +46689,7 @@
         <v>1972.7</v>
       </c>
       <c r="J8">
-        <v>14.46</v>
+        <v>24.23</v>
       </c>
       <c r="K8">
         <v>2090</v>

</xml_diff>

<commit_message>
refactor: apply Zelazny charting rules
- Change relative KPIs (Mietsteigerung, maintSqm, unitsPerEmp) to line charts
- Differentiate trend variables (lines) from absolute volumes (bars)
- Rebuilt export files
</commit_message>
<xml_diff>
--- a/Vonovia_Dashboard.xlsx
+++ b/Vonovia_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/08ec859eac6fe40e/ControllingDashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{0911EDB5-7703-9444-BB60-64BDA88E5045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF323A7C-09FD-714B-A12A-8FC384D8CAFD}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{0911EDB5-7703-9444-BB60-64BDA88E5045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F007BC10-93DF-6040-82A0-8DBDE57A125F}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{B42F3329-DB07-034F-B293-586B02AD4095}"/>
   </bookViews>
@@ -229,13 +229,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <numFmt numFmtId="35" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="35" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <numFmt numFmtId="35" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
@@ -310,12 +304,12 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Dashboard" pivot="0" table="0" count="10" xr9:uid="{3B652199-5835-A642-A53B-64313F011CA3}">
+      <tableStyleElement type="wholeTable" dxfId="5"/>
+      <tableStyleElement type="headerRow" dxfId="4"/>
+    </tableStyle>
+    <tableStyle name="SlicerStyleDark1 2" pivot="0" table="0" count="10" xr9:uid="{5472629C-5CA3-B047-A9E0-DF147B435016}">
       <tableStyleElement type="wholeTable" dxfId="7"/>
       <tableStyleElement type="headerRow" dxfId="6"/>
-    </tableStyle>
-    <tableStyle name="SlicerStyleDark1 2" pivot="0" table="0" count="10" xr9:uid="{5472629C-5CA3-B047-A9E0-DF147B435016}">
-      <tableStyleElement type="wholeTable" dxfId="9"/>
-      <tableStyleElement type="headerRow" dxfId="8"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -45988,12 +45982,12 @@
     <tableColumn id="6" xr3:uid="{0664C52D-2560-B041-AC8B-DB8A6D0FA61C}" name="Kundenzufriedenheit (CSI) in %"/>
     <tableColumn id="7" xr3:uid="{805F5C45-B6C1-164C-A47F-0C2F456D2451}" name="Leerstandsquote in %"/>
     <tableColumn id="8" xr3:uid="{632C0AA5-98D6-2247-AFC3-908E345F6ECC}" name="Mietsteigerung organisch in %"/>
-    <tableColumn id="9" xr3:uid="{5B26CC56-9C2A-CD42-BC7F-9A4101395461}" name="Gesamtsumme Instandhaltung/Modernisierung" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{5B26CC56-9C2A-CD42-BC7F-9A4101395461}" name="Gesamtsumme Instandhaltung/Modernisierung" dataDxfId="3"/>
     <tableColumn id="10" xr3:uid="{8F0E2C95-6963-6349-8EA6-64702ED9A5B9}" name="Instandhaltungsaufwand (€/m²)"/>
     <tableColumn id="11" xr3:uid="{51BE30B4-8E11-AB4E-893F-19568DEC1F7B}" name="Anzahl neu gebauter Einheiten"/>
     <tableColumn id="12" xr3:uid="{2EC3FDD8-4F36-834D-A011-A776F6314EAF}" name="CO₂-Intensität in kg CO₂e/m²"/>
     <tableColumn id="13" xr3:uid="{EB245DE4-A3F2-CF4C-BD13-2177FE1C4006}" name="Mitarbeiterzufriedenheit"/>
-    <tableColumn id="14" xr3:uid="{4CFC06F0-9445-2541-B310-01F9C4940F7F}" name="Bewirtschaftete Einheiten pro Mitarbeiter" dataDxfId="4"/>
+    <tableColumn id="14" xr3:uid="{4CFC06F0-9445-2541-B310-01F9C4940F7F}" name="Bewirtschaftete Einheiten pro Mitarbeiter" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -46704,12 +46698,104 @@
         <v>47.8</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="I12"/>
+      <c r="N12"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="I13"/>
+      <c r="N13"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="I14"/>
+      <c r="N14"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="I15"/>
+      <c r="N15"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="I16"/>
+      <c r="N16"/>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I17"/>
+      <c r="N17"/>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I18"/>
+      <c r="N18"/>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I19"/>
+      <c r="N19"/>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B20" s="1"/>
+      <c r="I20"/>
+      <c r="N20"/>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I21"/>
+      <c r="N21"/>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I22"/>
+      <c r="N22"/>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I23"/>
+      <c r="N23"/>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I24"/>
+      <c r="N24"/>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I25"/>
+      <c r="N25"/>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I26"/>
+      <c r="N26"/>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I27"/>
+      <c r="N27"/>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I28"/>
+      <c r="N28"/>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I29"/>
+      <c r="N29"/>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I30"/>
+      <c r="N30"/>
+    </row>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I31"/>
+      <c r="N31"/>
+    </row>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I32"/>
+      <c r="N32"/>
+    </row>
+    <row r="33" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I33"/>
+      <c r="N33"/>
+    </row>
+    <row r="34" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="I34"/>
+      <c r="N34"/>
+    </row>
+    <row r="35" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
+      <c r="I35"/>
+      <c r="N35"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>